<commit_message>
Auto update Pengadaan 2026-09-03 08:08:16
</commit_message>
<xml_diff>
--- a/output/tepra/2026/Tepra Kobar_Progres PBJ tahun 2026 (2026-09-03).xlsx
+++ b/output/tepra/2026/Tepra Kobar_Progres PBJ tahun 2026 (2026-09-03).xlsx
@@ -1267,22 +1267,22 @@
         <v>304521329</v>
       </c>
       <c r="E25" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F25" s="6" t="n">
-        <v>98994684</v>
+        <v>108974684</v>
       </c>
       <c r="G25" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H25" s="6" t="n">
-        <v>51881289</v>
+        <v>52571289</v>
       </c>
       <c r="I25" s="4" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="J25" s="6" t="n">
-        <v>205526645</v>
+        <v>195546645</v>
       </c>
     </row>
     <row r="26" ht="45" customHeight="1">
@@ -2877,22 +2877,22 @@
         <v>32552221446</v>
       </c>
       <c r="E67" s="12" t="n">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="F67" s="13" t="n">
-        <v>6186288817</v>
+        <v>6196268817</v>
       </c>
       <c r="G67" s="12" t="n">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="H67" s="13" t="n">
-        <v>5722240158.6</v>
+        <v>5722930158.6</v>
       </c>
       <c r="I67" s="12" t="n">
-        <v>3553</v>
+        <v>3552</v>
       </c>
       <c r="J67" s="13" t="n">
-        <v>26365932629</v>
+        <v>26355952629</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto update Pengadaan 2026-09-03 10:09:52
</commit_message>
<xml_diff>
--- a/output/tepra/2026/Tepra Kobar_Progres PBJ tahun 2026 (2026-09-03).xlsx
+++ b/output/tepra/2026/Tepra Kobar_Progres PBJ tahun 2026 (2026-09-03).xlsx
@@ -989,22 +989,22 @@
         </is>
       </c>
       <c r="C17" s="4" t="n">
-        <v>103</v>
+        <v>126</v>
       </c>
       <c r="D17" s="6" t="n">
         <v>677290237</v>
       </c>
       <c r="E17" s="4" t="n">
-        <v>13</v>
+        <v>36</v>
       </c>
       <c r="F17" s="6" t="n">
         <v>137583844</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>13</v>
+        <v>36</v>
       </c>
       <c r="H17" s="6" t="n">
-        <v>116218702</v>
+        <v>1301651478</v>
       </c>
       <c r="I17" s="4" t="n">
         <v>90</v>
@@ -1125,22 +1125,22 @@
         </is>
       </c>
       <c r="C21" s="4" t="n">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="D21" s="6" t="n">
-        <v>2245544792</v>
+        <v>2236040639</v>
       </c>
       <c r="E21" s="4" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F21" s="6" t="n">
-        <v>1136240668</v>
+        <v>1126736515</v>
       </c>
       <c r="G21" s="4" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="H21" s="6" t="n">
-        <v>1115612710.6</v>
+        <v>2912112710.6</v>
       </c>
       <c r="I21" s="4" t="n">
         <v>129</v>
@@ -1468,13 +1468,13 @@
         <v>112</v>
       </c>
       <c r="D31" s="6" t="n">
-        <v>1305525621</v>
+        <v>1279995621</v>
       </c>
       <c r="E31" s="4" t="n">
         <v>10</v>
       </c>
       <c r="F31" s="6" t="n">
-        <v>280944208</v>
+        <v>255414208</v>
       </c>
       <c r="G31" s="4" t="n">
         <v>10</v>
@@ -1635,25 +1635,25 @@
         </is>
       </c>
       <c r="C36" s="8" t="n">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="D36" s="10" t="n">
         <v>282819298</v>
       </c>
       <c r="E36" s="8" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="F36" s="10" t="n">
         <v>141795000</v>
       </c>
       <c r="G36" s="8" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H36" s="10" t="n">
-        <v>64745634</v>
+        <v>76907682</v>
       </c>
       <c r="I36" s="8" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="J36" s="10" t="n">
         <v>141024298</v>
@@ -2871,25 +2871,25 @@
         </is>
       </c>
       <c r="C67" s="12" t="n">
-        <v>3932</v>
+        <v>3959</v>
       </c>
       <c r="D67" s="13" t="n">
-        <v>32552221446</v>
+        <v>32517187293</v>
       </c>
       <c r="E67" s="12" t="n">
-        <v>380</v>
+        <v>406</v>
       </c>
       <c r="F67" s="13" t="n">
-        <v>6196268817</v>
+        <v>6161234664</v>
       </c>
       <c r="G67" s="12" t="n">
-        <v>380</v>
+        <v>406</v>
       </c>
       <c r="H67" s="13" t="n">
-        <v>5722930158.6</v>
+        <v>8717024982.6</v>
       </c>
       <c r="I67" s="12" t="n">
-        <v>3552</v>
+        <v>3553</v>
       </c>
       <c r="J67" s="13" t="n">
         <v>26355952629</v>
@@ -4596,28 +4596,28 @@
         </is>
       </c>
       <c r="C36" s="8" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D36" s="10" t="n">
-        <v>595373450</v>
+        <v>379426400</v>
       </c>
       <c r="E36" s="8" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F36" s="10" t="n">
-        <v>345935300</v>
+        <v>201970600</v>
       </c>
       <c r="G36" s="8" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H36" s="10" t="n">
-        <v>154581508</v>
+        <v>142419460</v>
       </c>
       <c r="I36" s="8" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J36" s="10" t="n">
-        <v>154581508</v>
+        <v>142419460</v>
       </c>
       <c r="K36" s="11" t="inlineStr">
         <is>
@@ -4630,10 +4630,10 @@
         </is>
       </c>
       <c r="M36" s="8" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N36" s="10" t="n">
-        <v>249438150</v>
+        <v>177455800</v>
       </c>
     </row>
     <row r="37" ht="45" customHeight="1">
@@ -6408,28 +6408,28 @@
         </is>
       </c>
       <c r="C67" s="12" t="n">
-        <v>809</v>
+        <v>806</v>
       </c>
       <c r="D67" s="13" t="n">
-        <v>95882716294</v>
+        <v>95666769244</v>
       </c>
       <c r="E67" s="12" t="n">
-        <v>492</v>
+        <v>490</v>
       </c>
       <c r="F67" s="13" t="n">
-        <v>62675975663</v>
+        <v>62532010963</v>
       </c>
       <c r="G67" s="12" t="n">
-        <v>492</v>
+        <v>490</v>
       </c>
       <c r="H67" s="13" t="n">
-        <v>60673958430.41</v>
+        <v>60661796382.41</v>
       </c>
       <c r="I67" s="12" t="n">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="J67" s="13" t="n">
-        <v>28562577087</v>
+        <v>28550415039</v>
       </c>
       <c r="K67" s="12" t="n">
         <v>7</v>
@@ -6438,10 +6438,10 @@
         <v>513626623</v>
       </c>
       <c r="M67" s="12" t="n">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="N67" s="13" t="n">
-        <v>33206740631</v>
+        <v>33134758281</v>
       </c>
     </row>
   </sheetData>
@@ -7231,34 +7231,34 @@
         </is>
       </c>
       <c r="C17" s="4" t="n">
-        <v>34</v>
+        <v>11</v>
       </c>
       <c r="D17" s="6" t="n">
-        <v>49873115767</v>
+        <v>7521643942</v>
       </c>
       <c r="E17" s="4" t="n">
-        <v>33</v>
+        <v>10</v>
       </c>
       <c r="F17" s="6" t="n">
-        <v>49502018488</v>
+        <v>7150546663</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>33</v>
+        <v>10</v>
       </c>
       <c r="H17" s="6" t="n">
-        <v>5975304750</v>
+        <v>4789871974</v>
       </c>
       <c r="I17" s="4" t="n">
-        <v>33</v>
+        <v>10</v>
       </c>
       <c r="J17" s="6" t="n">
-        <v>5975304750</v>
+        <v>4789871974</v>
       </c>
       <c r="K17" s="4" t="n">
-        <v>24</v>
+        <v>3</v>
       </c>
       <c r="L17" s="6" t="n">
-        <v>1997011203</v>
+        <v>906164395</v>
       </c>
       <c r="M17" s="4" t="n">
         <v>1</v>
@@ -7451,28 +7451,28 @@
         </is>
       </c>
       <c r="C21" s="4" t="n">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D21" s="6" t="n">
-        <v>38006848385</v>
+        <v>36557914658</v>
       </c>
       <c r="E21" s="4" t="n">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="F21" s="6" t="n">
-        <v>32261200833</v>
+        <v>30812267106</v>
       </c>
       <c r="G21" s="4" t="n">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H21" s="6" t="n">
-        <v>32168354970</v>
+        <v>30371854970</v>
       </c>
       <c r="I21" s="4" t="n">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="J21" s="6" t="n">
-        <v>31161310970</v>
+        <v>29364810970</v>
       </c>
       <c r="K21" s="7" t="inlineStr">
         <is>
@@ -8044,13 +8044,13 @@
         <v>11</v>
       </c>
       <c r="D32" s="10" t="n">
-        <v>4274621970</v>
+        <v>3639664785</v>
       </c>
       <c r="E32" s="8" t="n">
         <v>10</v>
       </c>
       <c r="F32" s="10" t="n">
-        <v>3786710370</v>
+        <v>3151753185</v>
       </c>
       <c r="G32" s="8" t="n">
         <v>10</v>
@@ -10285,34 +10285,34 @@
         </is>
       </c>
       <c r="C67" s="12" t="n">
-        <v>232</v>
+        <v>208</v>
       </c>
       <c r="D67" s="13" t="n">
-        <v>177388972233</v>
+        <v>132953609496</v>
       </c>
       <c r="E67" s="12" t="n">
-        <v>152</v>
+        <v>128</v>
       </c>
       <c r="F67" s="13" t="n">
-        <v>139525277778</v>
+        <v>95089915041</v>
       </c>
       <c r="G67" s="12" t="n">
-        <v>152</v>
+        <v>128</v>
       </c>
       <c r="H67" s="13" t="n">
-        <v>65283438800.98</v>
+        <v>62301506024.98</v>
       </c>
       <c r="I67" s="12" t="n">
-        <v>133</v>
+        <v>109</v>
       </c>
       <c r="J67" s="13" t="n">
-        <v>61224505000.97</v>
+        <v>58242572224.97</v>
       </c>
       <c r="K67" s="12" t="n">
-        <v>29</v>
+        <v>8</v>
       </c>
       <c r="L67" s="13" t="n">
-        <v>3046617077</v>
+        <v>1955770269</v>
       </c>
       <c r="M67" s="12" t="n">
         <v>80</v>

</xml_diff>

<commit_message>
Auto update Pengadaan 2026-09-03 12:08:31
</commit_message>
<xml_diff>
--- a/output/tepra/2026/Tepra Kobar_Progres PBJ tahun 2026 (2026-09-03).xlsx
+++ b/output/tepra/2026/Tepra Kobar_Progres PBJ tahun 2026 (2026-09-03).xlsx
@@ -989,22 +989,22 @@
         </is>
       </c>
       <c r="C17" s="4" t="n">
-        <v>126</v>
+        <v>103</v>
       </c>
       <c r="D17" s="6" t="n">
         <v>677290237</v>
       </c>
       <c r="E17" s="4" t="n">
-        <v>36</v>
+        <v>13</v>
       </c>
       <c r="F17" s="6" t="n">
         <v>137583844</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>36</v>
+        <v>13</v>
       </c>
       <c r="H17" s="6" t="n">
-        <v>1301651478</v>
+        <v>116218702</v>
       </c>
       <c r="I17" s="4" t="n">
         <v>90</v>
@@ -1125,22 +1125,22 @@
         </is>
       </c>
       <c r="C21" s="4" t="n">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="D21" s="6" t="n">
-        <v>2236040639</v>
+        <v>2245544792</v>
       </c>
       <c r="E21" s="4" t="n">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F21" s="6" t="n">
-        <v>1126736515</v>
+        <v>1136240668</v>
       </c>
       <c r="G21" s="4" t="n">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="H21" s="6" t="n">
-        <v>2912112710.6</v>
+        <v>1115612710.6</v>
       </c>
       <c r="I21" s="4" t="n">
         <v>129</v>
@@ -1468,13 +1468,13 @@
         <v>112</v>
       </c>
       <c r="D31" s="6" t="n">
-        <v>1279995621</v>
+        <v>1305525621</v>
       </c>
       <c r="E31" s="4" t="n">
         <v>10</v>
       </c>
       <c r="F31" s="6" t="n">
-        <v>255414208</v>
+        <v>280944208</v>
       </c>
       <c r="G31" s="4" t="n">
         <v>10</v>
@@ -1635,25 +1635,25 @@
         </is>
       </c>
       <c r="C36" s="8" t="n">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="D36" s="10" t="n">
         <v>282819298</v>
       </c>
       <c r="E36" s="8" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F36" s="10" t="n">
         <v>141795000</v>
       </c>
       <c r="G36" s="8" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H36" s="10" t="n">
-        <v>76907682</v>
+        <v>64745634</v>
       </c>
       <c r="I36" s="8" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="J36" s="10" t="n">
         <v>141024298</v>
@@ -2871,25 +2871,25 @@
         </is>
       </c>
       <c r="C67" s="12" t="n">
-        <v>3959</v>
+        <v>3932</v>
       </c>
       <c r="D67" s="13" t="n">
-        <v>32517187293</v>
+        <v>32552221446</v>
       </c>
       <c r="E67" s="12" t="n">
-        <v>406</v>
+        <v>380</v>
       </c>
       <c r="F67" s="13" t="n">
-        <v>6161234664</v>
+        <v>6196268817</v>
       </c>
       <c r="G67" s="12" t="n">
-        <v>406</v>
+        <v>380</v>
       </c>
       <c r="H67" s="13" t="n">
-        <v>8717024982.6</v>
+        <v>5722930158.6</v>
       </c>
       <c r="I67" s="12" t="n">
-        <v>3553</v>
+        <v>3552</v>
       </c>
       <c r="J67" s="13" t="n">
         <v>26355952629</v>
@@ -4596,28 +4596,28 @@
         </is>
       </c>
       <c r="C36" s="8" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="D36" s="10" t="n">
-        <v>379426400</v>
+        <v>595373450</v>
       </c>
       <c r="E36" s="8" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F36" s="10" t="n">
-        <v>201970600</v>
+        <v>345935300</v>
       </c>
       <c r="G36" s="8" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H36" s="10" t="n">
-        <v>142419460</v>
+        <v>154581508</v>
       </c>
       <c r="I36" s="8" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J36" s="10" t="n">
-        <v>142419460</v>
+        <v>154581508</v>
       </c>
       <c r="K36" s="11" t="inlineStr">
         <is>
@@ -4630,10 +4630,10 @@
         </is>
       </c>
       <c r="M36" s="8" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N36" s="10" t="n">
-        <v>177455800</v>
+        <v>249438150</v>
       </c>
     </row>
     <row r="37" ht="45" customHeight="1">
@@ -6408,28 +6408,28 @@
         </is>
       </c>
       <c r="C67" s="12" t="n">
-        <v>806</v>
+        <v>809</v>
       </c>
       <c r="D67" s="13" t="n">
-        <v>95666769244</v>
+        <v>95882716294</v>
       </c>
       <c r="E67" s="12" t="n">
-        <v>490</v>
+        <v>492</v>
       </c>
       <c r="F67" s="13" t="n">
-        <v>62532010963</v>
+        <v>62675975663</v>
       </c>
       <c r="G67" s="12" t="n">
-        <v>490</v>
+        <v>492</v>
       </c>
       <c r="H67" s="13" t="n">
-        <v>60661796382.41</v>
+        <v>60673958430.41</v>
       </c>
       <c r="I67" s="12" t="n">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="J67" s="13" t="n">
-        <v>28550415039</v>
+        <v>28562577087</v>
       </c>
       <c r="K67" s="12" t="n">
         <v>7</v>
@@ -6438,10 +6438,10 @@
         <v>513626623</v>
       </c>
       <c r="M67" s="12" t="n">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="N67" s="13" t="n">
-        <v>33134758281</v>
+        <v>33206740631</v>
       </c>
     </row>
   </sheetData>
@@ -7231,34 +7231,34 @@
         </is>
       </c>
       <c r="C17" s="4" t="n">
-        <v>11</v>
+        <v>34</v>
       </c>
       <c r="D17" s="6" t="n">
-        <v>7521643942</v>
+        <v>49873115767</v>
       </c>
       <c r="E17" s="4" t="n">
-        <v>10</v>
+        <v>33</v>
       </c>
       <c r="F17" s="6" t="n">
-        <v>7150546663</v>
+        <v>49502018488</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>10</v>
+        <v>33</v>
       </c>
       <c r="H17" s="6" t="n">
-        <v>4789871974</v>
+        <v>5975304750</v>
       </c>
       <c r="I17" s="4" t="n">
-        <v>10</v>
+        <v>33</v>
       </c>
       <c r="J17" s="6" t="n">
-        <v>4789871974</v>
+        <v>5975304750</v>
       </c>
       <c r="K17" s="4" t="n">
-        <v>3</v>
+        <v>24</v>
       </c>
       <c r="L17" s="6" t="n">
-        <v>906164395</v>
+        <v>1997011203</v>
       </c>
       <c r="M17" s="4" t="n">
         <v>1</v>
@@ -7451,28 +7451,28 @@
         </is>
       </c>
       <c r="C21" s="4" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D21" s="6" t="n">
-        <v>36557914658</v>
+        <v>38006848385</v>
       </c>
       <c r="E21" s="4" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="F21" s="6" t="n">
-        <v>30812267106</v>
+        <v>32261200833</v>
       </c>
       <c r="G21" s="4" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="H21" s="6" t="n">
-        <v>30371854970</v>
+        <v>32168354970</v>
       </c>
       <c r="I21" s="4" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="J21" s="6" t="n">
-        <v>29364810970</v>
+        <v>31161310970</v>
       </c>
       <c r="K21" s="7" t="inlineStr">
         <is>
@@ -8044,13 +8044,13 @@
         <v>11</v>
       </c>
       <c r="D32" s="10" t="n">
-        <v>3639664785</v>
+        <v>4274621970</v>
       </c>
       <c r="E32" s="8" t="n">
         <v>10</v>
       </c>
       <c r="F32" s="10" t="n">
-        <v>3151753185</v>
+        <v>3786710370</v>
       </c>
       <c r="G32" s="8" t="n">
         <v>10</v>
@@ -10285,34 +10285,34 @@
         </is>
       </c>
       <c r="C67" s="12" t="n">
-        <v>208</v>
+        <v>232</v>
       </c>
       <c r="D67" s="13" t="n">
-        <v>132953609496</v>
+        <v>177388972233</v>
       </c>
       <c r="E67" s="12" t="n">
-        <v>128</v>
+        <v>152</v>
       </c>
       <c r="F67" s="13" t="n">
-        <v>95089915041</v>
+        <v>139525277778</v>
       </c>
       <c r="G67" s="12" t="n">
-        <v>128</v>
+        <v>152</v>
       </c>
       <c r="H67" s="13" t="n">
-        <v>62301506024.98</v>
+        <v>65283438800.98</v>
       </c>
       <c r="I67" s="12" t="n">
-        <v>109</v>
+        <v>133</v>
       </c>
       <c r="J67" s="13" t="n">
-        <v>58242572224.97</v>
+        <v>61224505000.97</v>
       </c>
       <c r="K67" s="12" t="n">
-        <v>8</v>
+        <v>29</v>
       </c>
       <c r="L67" s="13" t="n">
-        <v>1955770269</v>
+        <v>3046617077</v>
       </c>
       <c r="M67" s="12" t="n">
         <v>80</v>

</xml_diff>